<commit_message>
TAREFA 09 parcialmente concluída
</commit_message>
<xml_diff>
--- a/Avancado/09 - Funções de data e hora.xlsx
+++ b/Avancado/09 - Funções de data e hora.xlsx
@@ -1,15 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DD411B-DD67-46CB-BF9F-FC19FFA2CA59}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Funções de data 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Funções de data 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Funções de hora" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,9 +26,72 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>Amália</t>
+  </si>
+  <si>
+    <t>Bruno</t>
+  </si>
+  <si>
+    <t>Duarte</t>
+  </si>
+  <si>
+    <t>Eduardo</t>
+  </si>
+  <si>
+    <t>Roberta</t>
+  </si>
+  <si>
+    <t>Rodrigo</t>
+  </si>
+  <si>
+    <t>FUNÇÕES DE DATA</t>
+  </si>
+  <si>
+    <t>NOME</t>
+  </si>
+  <si>
+    <t>DATA DE NASCIMENTO</t>
+  </si>
+  <si>
+    <t>ANO</t>
+  </si>
+  <si>
+    <t>MÊS</t>
+  </si>
+  <si>
+    <t>DIA</t>
+  </si>
+  <si>
+    <t>IDADE</t>
+  </si>
+  <si>
+    <t>Nº DE DIAS VIVIDOS</t>
+  </si>
+  <si>
+    <t>Funções de data e hora</t>
+  </si>
+  <si>
+    <t>Hoje</t>
+  </si>
+  <si>
+    <t>Agora</t>
+  </si>
+  <si>
+    <t>Data completa</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="171" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="172" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +99,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +130,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +462,295 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4">
+        <v>23525</v>
+      </c>
+      <c r="C3" s="5">
+        <f>YEAR(B3)</f>
+        <v>1964</v>
+      </c>
+      <c r="D3" s="5">
+        <f>MONTH(B3)</f>
+        <v>5</v>
+      </c>
+      <c r="E3" s="5">
+        <f>DAY(B3)</f>
+        <v>28</v>
+      </c>
+      <c r="F3" s="6">
+        <f ca="1">ROUNDDOWN((TODAY()-B3)/365.25,0)</f>
+        <v>61</v>
+      </c>
+      <c r="G3" s="7">
+        <f ca="1">TODAY()-B3</f>
+        <v>22566</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4">
+        <v>30647</v>
+      </c>
+      <c r="C4" s="5">
+        <f t="shared" ref="C4:C8" si="0">YEAR(B4)</f>
+        <v>1983</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" ref="D4:D8" si="1">MONTH(B4)</f>
+        <v>11</v>
+      </c>
+      <c r="E4" s="5">
+        <f t="shared" ref="E4:E8" si="2">DAY(B4)</f>
+        <v>27</v>
+      </c>
+      <c r="F4" s="6">
+        <f t="shared" ref="F4:F8" ca="1" si="3">ROUNDDOWN((TODAY()-B4)/365.25,0)</f>
+        <v>42</v>
+      </c>
+      <c r="G4" s="7">
+        <f t="shared" ref="G4:G8" ca="1" si="4">TODAY()-B4</f>
+        <v>15444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4">
+        <v>25727</v>
+      </c>
+      <c r="C5" s="5">
+        <f t="shared" si="0"/>
+        <v>1970</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="E5" s="5">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="F5" s="6">
+        <f t="shared" ca="1" si="3"/>
+        <v>55</v>
+      </c>
+      <c r="G5" s="7">
+        <f t="shared" ca="1" si="4"/>
+        <v>20364</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4">
+        <v>41011</v>
+      </c>
+      <c r="C6" s="5">
+        <f t="shared" si="0"/>
+        <v>2012</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="E6" s="5">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F6" s="6">
+        <f t="shared" ca="1" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="shared" ca="1" si="4"/>
+        <v>5080</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4">
+        <v>42617</v>
+      </c>
+      <c r="C7" s="5">
+        <f t="shared" si="0"/>
+        <v>2016</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="E7" s="5">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="F7" s="6">
+        <f t="shared" ca="1" si="3"/>
+        <v>9</v>
+      </c>
+      <c r="G7" s="7">
+        <f t="shared" ca="1" si="4"/>
+        <v>3474</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4">
+        <v>27264</v>
+      </c>
+      <c r="C8" s="5">
+        <f t="shared" si="0"/>
+        <v>1974</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="E8" s="5">
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+      <c r="F8" s="6">
+        <f t="shared" ca="1" si="3"/>
+        <v>51</v>
+      </c>
+      <c r="G8" s="7">
+        <f t="shared" ca="1" si="4"/>
+        <v>18827</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DFC884-D6D9-4513-800E-0A9DA5576FE5}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="10">
+        <f ca="1">TODAY()</f>
+        <v>46091</v>
+      </c>
+      <c r="C3" s="13">
+        <f ca="1">MONTH(B3)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="12">
+        <f ca="1">NOW()</f>
+        <v>46091.91243773148</v>
+      </c>
+      <c r="C4" s="14"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="11">
+        <f ca="1">TODAY()</f>
+        <v>46091</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B5:D5"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="B4" formula="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58EDC447-FA2C-4B58-B3E9-F7C37B1141E6}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
atividade 09 parcialmente concluida
</commit_message>
<xml_diff>
--- a/Avancado/09 - Funções de data e hora.xlsx
+++ b/Avancado/09 - Funções de data e hora.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DD411B-DD67-46CB-BF9F-FC19FFA2CA59}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A461C3-9F85-4186-97FB-196BD2C7CE87}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,8 +88,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="171" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="172" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -155,34 +155,34 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,15 +472,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -509,26 +509,26 @@
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>23525</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <f>YEAR(B3)</f>
         <v>1964</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="4">
         <f>MONTH(B3)</f>
         <v>5</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="4">
         <f>DAY(B3)</f>
         <v>28</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <f ca="1">ROUNDDOWN((TODAY()-B3)/365.25,0)</f>
         <v>61</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="6">
         <f ca="1">TODAY()-B3</f>
         <v>22566</v>
       </c>
@@ -537,26 +537,26 @@
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>30647</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <f t="shared" ref="C4:C8" si="0">YEAR(B4)</f>
         <v>1983</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <f t="shared" ref="D4:D8" si="1">MONTH(B4)</f>
         <v>11</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <f t="shared" ref="E4:E8" si="2">DAY(B4)</f>
         <v>27</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <f t="shared" ref="F4:F8" ca="1" si="3">ROUNDDOWN((TODAY()-B4)/365.25,0)</f>
         <v>42</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="6">
         <f t="shared" ref="G4:G8" ca="1" si="4">TODAY()-B4</f>
         <v>15444</v>
       </c>
@@ -565,26 +565,26 @@
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>25727</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <f t="shared" si="0"/>
         <v>1970</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <f t="shared" ca="1" si="3"/>
         <v>55</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="6">
         <f t="shared" ca="1" si="4"/>
         <v>20364</v>
       </c>
@@ -593,26 +593,26 @@
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>41011</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <f t="shared" si="0"/>
         <v>2012</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <f t="shared" ca="1" si="3"/>
         <v>13</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="6">
         <f t="shared" ca="1" si="4"/>
         <v>5080</v>
       </c>
@@ -621,26 +621,26 @@
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>42617</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <f t="shared" si="0"/>
         <v>2016</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <f t="shared" ca="1" si="3"/>
         <v>9</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="6">
         <f t="shared" ca="1" si="4"/>
         <v>3474</v>
       </c>
@@ -649,26 +649,26 @@
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>27264</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <f t="shared" si="0"/>
         <v>1974</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <f t="shared" si="2"/>
         <v>23</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <f t="shared" ca="1" si="3"/>
         <v>51</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="6">
         <f t="shared" ca="1" si="4"/>
         <v>18827</v>
       </c>
@@ -692,22 +692,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="7">
         <f ca="1">TODAY()</f>
         <v>46091</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="9">
         <f ca="1">MONTH(B3)</f>
         <v>3</v>
       </c>
@@ -716,22 +716,22 @@
       <c r="A4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="8">
         <f ca="1">NOW()</f>
-        <v>46091.91243773148</v>
-      </c>
-      <c r="C4" s="14"/>
+        <v>46091.916796527781</v>
+      </c>
+      <c r="C4" s="10"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="14">
         <f ca="1">TODAY()</f>
         <v>46091</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
TAREFA 09 parcialmente concluída; quase lá
</commit_message>
<xml_diff>
--- a/Avancado/09 - Funções de data e hora.xlsx
+++ b/Avancado/09 - Funções de data e hora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49A461C3-9F85-4186-97FB-196BD2C7CE87}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CA9AC7-9ECC-4360-B17D-E90EAB24F072}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Funções de data 1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Amália</t>
   </si>
@@ -81,6 +81,42 @@
   </si>
   <si>
     <t>Data completa</t>
+  </si>
+  <si>
+    <t>Dia</t>
+  </si>
+  <si>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t>Meu nascimento</t>
+  </si>
+  <si>
+    <t>Dias vividos</t>
+  </si>
+  <si>
+    <t>Meses Vividos</t>
+  </si>
+  <si>
+    <t>Anos vividos</t>
+  </si>
+  <si>
+    <t>Exemplo</t>
+  </si>
+  <si>
+    <t>Hora</t>
+  </si>
+  <si>
+    <t>Minto</t>
+  </si>
+  <si>
+    <t>Segundo</t>
+  </si>
+  <si>
+    <t>Tempo</t>
   </si>
 </sst>
 </file>
@@ -89,7 +125,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="170" formatCode="[$-416]mmmm&quot;-&quot;yy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -149,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -161,16 +197,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -180,8 +209,34 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,15 +527,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -525,12 +580,12 @@
         <v>28</v>
       </c>
       <c r="F3" s="5">
-        <f ca="1">ROUNDDOWN((TODAY()-B3)/365.25,0)</f>
+        <f ca="1">TRUNC((TODAY()-B3)/365.25,0)</f>
         <v>61</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="5">
         <f ca="1">TODAY()-B3</f>
-        <v>22566</v>
+        <v>22567</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -553,12 +608,12 @@
         <v>27</v>
       </c>
       <c r="F4" s="5">
-        <f t="shared" ref="F4:F8" ca="1" si="3">ROUNDDOWN((TODAY()-B4)/365.25,0)</f>
+        <f t="shared" ref="F4:F8" ca="1" si="3">TRUNC((TODAY()-B4)/365.25,0)</f>
         <v>42</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <f t="shared" ref="G4:G8" ca="1" si="4">TODAY()-B4</f>
-        <v>15444</v>
+        <v>15445</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -584,9 +639,9 @@
         <f t="shared" ca="1" si="3"/>
         <v>55</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>20364</v>
+        <v>20365</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -612,9 +667,9 @@
         <f t="shared" ca="1" si="3"/>
         <v>13</v>
       </c>
-      <c r="G6" s="6">
-        <f t="shared" ca="1" si="4"/>
-        <v>5080</v>
+      <c r="G6" s="5">
+        <f ca="1">TODAY()-B6</f>
+        <v>5081</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -640,9 +695,9 @@
         <f t="shared" ca="1" si="3"/>
         <v>9</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>3474</v>
+        <v>3475</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -668,9 +723,9 @@
         <f t="shared" ca="1" si="3"/>
         <v>51</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>18827</v>
+        <v>18828</v>
       </c>
     </row>
   </sheetData>
@@ -683,55 +738,122 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22DFC884-D6D9-4513-800E-0A9DA5576FE5}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="3">
         <f ca="1">TODAY()</f>
-        <v>46091</v>
-      </c>
-      <c r="C3" s="9">
+        <v>46092</v>
+      </c>
+      <c r="C3" s="11">
+        <f ca="1">DATE(YEAR(B3),MONTH(B3),DAY(B3))</f>
+        <v>46092</v>
+      </c>
+      <c r="D3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="12">
+        <f ca="1">NOW()</f>
+        <v>46092.841347106485</v>
+      </c>
+      <c r="C4" s="13">
+        <f ca="1">TIME(HOUR(B4),MINUTE(B4),SECOND(B4))</f>
+        <v>0.8413425925925927</v>
+      </c>
+      <c r="D4" s="14">
+        <f ca="1">TIME(HOUR(B4),MINUTE(B4),SECOND(B4))</f>
+        <v>0.8413425925925927</v>
+      </c>
+      <c r="F4" s="10"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="15">
+        <f ca="1">TODAY()</f>
+        <v>46092</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="4">
+        <f ca="1">DAY(B3)</f>
+        <v>11</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="17">
+        <v>38965</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="4">
         <f ca="1">MONTH(B3)</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="8">
-        <f ca="1">NOW()</f>
-        <v>46091.916796527781</v>
-      </c>
-      <c r="C4" s="10"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="14">
-        <f ca="1">TODAY()</f>
-        <v>46091</v>
-      </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
+      <c r="D8" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="5">
+        <f ca="1">_xlfn.DAYS(NOW(),E7)</f>
+        <v>7127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4">
+        <f ca="1">YEAR(B3)</f>
+        <v>2026</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="4">
+        <f ca="1" xml:space="preserve"> (YEAR(B3) - YEAR(E7)) * 12 + MONTH(B3) - MONTH(E7)</f>
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D10" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="4">
+        <f ca="1">TRUNC((TODAY()-E7)/365.25,0)</f>
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -748,9 +870,104 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58EDC447-FA2C-4B58-B3E9-F7C37B1141E6}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="21">
+        <f ca="1">TIME(HOUR(NOW()),MINUTE(NOW()),SECOND(NOW()))</f>
+        <v>0.8413425925925927</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="20"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="4">
+        <f ca="1">HOUR(NOW())</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="4">
+        <f ca="1">MINUTE(NOW())</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="4">
+        <f ca="1">SECOND(NOW())</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="21">
+        <f ca="1">TIME(HOUR(NOW()),MINUTE(NOW()),SECOND(NOW()))</f>
+        <v>0.8413425925925927</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="20"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="19"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="19"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="19"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="19"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TAREFAS DE FUNÇÕES DE TEXTO E DATA CONCLUÍDAS
</commit_message>
<xml_diff>
--- a/Avancado/09 - Funções de data e hora.xlsx
+++ b/Avancado/09 - Funções de data e hora.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9C7A779-C3E2-4A2B-981C-5E335A37FFA9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{609438DE-8339-4361-8D30-85388E2B643F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Funções de data 1" sheetId="1" r:id="rId1"/>
@@ -155,8 +155,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="170" formatCode="[$-416]mmmm&quot;-&quot;yy"/>
-    <numFmt numFmtId="174" formatCode="00"/>
+    <numFmt numFmtId="165" formatCode="[$-416]mmmm&quot;-&quot;yy"/>
+    <numFmt numFmtId="166" formatCode="00"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -231,22 +231,13 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -256,9 +247,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -272,7 +260,19 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -564,15 +564,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -622,7 +622,7 @@
       </c>
       <c r="G3" s="5">
         <f ca="1">TODAY()-B3</f>
-        <v>22567</v>
+        <v>22574</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -650,7 +650,7 @@
       </c>
       <c r="G4" s="5">
         <f t="shared" ref="G4:G8" ca="1" si="4">TODAY()-B4</f>
-        <v>15445</v>
+        <v>15452</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -678,7 +678,7 @@
       </c>
       <c r="G5" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>20365</v>
+        <v>20372</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -706,7 +706,7 @@
       </c>
       <c r="G6" s="5">
         <f ca="1">TODAY()-B6</f>
-        <v>5081</v>
+        <v>5088</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -734,7 +734,7 @@
       </c>
       <c r="G7" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>3475</v>
+        <v>3482</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -762,7 +762,7 @@
       </c>
       <c r="G8" s="5">
         <f t="shared" ca="1" si="4"/>
-        <v>18828</v>
+        <v>18835</v>
       </c>
     </row>
   </sheetData>
@@ -786,12 +786,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -799,83 +799,83 @@
       </c>
       <c r="B3" s="3">
         <f ca="1">TODAY()</f>
-        <v>46092</v>
-      </c>
-      <c r="C3" s="11">
+        <v>46099</v>
+      </c>
+      <c r="C3" s="8">
         <f ca="1">DATE(YEAR(B3),MONTH(B3),DAY(B3))</f>
-        <v>46092</v>
-      </c>
-      <c r="D3" s="9"/>
+        <v>46099</v>
+      </c>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="9">
         <f ca="1">NOW()</f>
-        <v>46092.863810995368</v>
-      </c>
-      <c r="C4" s="13">
+        <v>46099.889732175929</v>
+      </c>
+      <c r="C4" s="10">
         <f ca="1">TIME(HOUR(B4),MINUTE(B4),SECOND(B4))</f>
-        <v>0.86380787037037043</v>
-      </c>
-      <c r="D4" s="14">
+        <v>0.88973379629629623</v>
+      </c>
+      <c r="D4" s="11">
         <f ca="1">TIME(HOUR(B4),MINUTE(B4),SECOND(B4))</f>
-        <v>0.86380787037037043</v>
-      </c>
-      <c r="F4" s="10"/>
+        <v>0.88973379629629623</v>
+      </c>
+      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="23">
         <f ca="1">TODAY()</f>
-        <v>46092</v>
-      </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
+        <v>46099</v>
+      </c>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="12" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="4">
         <f ca="1">DAY(B3)</f>
-        <v>11</v>
-      </c>
-      <c r="D7" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="13">
         <v>38965</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="12" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="4">
         <f ca="1">MONTH(B3)</f>
         <v>3</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="12" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="5">
         <f ca="1">_xlfn.DAYS(NOW(),E7)</f>
-        <v>7127</v>
+        <v>7134</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="12" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="4">
         <f ca="1">YEAR(B3)</f>
         <v>2026</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="12" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="4">
@@ -884,7 +884,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="12" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="4">
@@ -915,180 +915,180 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="20">
+      <c r="B1" s="16">
         <f ca="1">TIME(HOUR(NOW()),MINUTE(NOW()),SECOND(NOW()))</f>
-        <v>0.86380787037037043</v>
+        <v>0.88973379629629623</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="19"/>
+      <c r="A2" s="15"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="14" t="s">
         <v>26</v>
       </c>
       <c r="B3" s="4">
         <f ca="1">HOUR(NOW())</f>
-        <v>20</v>
-      </c>
-      <c r="C3" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="18" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="14" t="s">
         <v>27</v>
       </c>
       <c r="B4" s="4">
         <f ca="1">MINUTE(NOW())</f>
-        <v>43</v>
-      </c>
-      <c r="C4" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="14" t="s">
         <v>28</v>
       </c>
       <c r="B5" s="4">
         <f ca="1">SECOND(NOW())</f>
-        <v>53</v>
-      </c>
-      <c r="C5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="16">
         <f ca="1">TIME(B3,B4,B5)</f>
-        <v>0.86380787037037043</v>
-      </c>
-      <c r="C6" s="22" t="s">
+        <v>0.88973379629629623</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
+      <c r="A7" s="15"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="21" t="s">
+      <c r="F8" s="17" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="16">
         <v>4.7789351851851847E-2</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="19">
         <f>HOUR(B9)</f>
         <v>1</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="19">
         <f>MINUTE(B9)</f>
         <v>8</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="19">
         <f>SECOND(B9)</f>
         <v>49</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="16">
         <f>TIME(C9,D9,E9)</f>
         <v>4.7789351851851847E-2</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="16">
         <v>4.0625000000000001E-2</v>
       </c>
-      <c r="C10" s="23">
+      <c r="C10" s="19">
         <f t="shared" ref="C10:C12" si="0">HOUR(B10)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="19">
         <f t="shared" ref="D10:D12" si="1">MINUTE(B10)</f>
         <v>58</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="19">
         <f t="shared" ref="E10:E12" si="2">SECOND(B10)</f>
         <v>30</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="16">
         <f t="shared" ref="F10:F12" si="3">TIME(C10,D10,E10)</f>
         <v>4.0625000000000001E-2</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="16">
         <v>4.1087962962962958E-2</v>
       </c>
-      <c r="C11" s="23">
+      <c r="C11" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="19">
         <f t="shared" si="1"/>
         <v>59</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="19">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="16">
         <f t="shared" si="3"/>
         <v>4.1087962962962958E-2</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="16">
         <v>4.5833333333333337E-2</v>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="19">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="19">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="16">
         <f t="shared" si="3"/>
         <v>4.5833333333333337E-2</v>
       </c>

</xml_diff>